<commit_message>
fix: limit cell formatting to Grade column only
</commit_message>
<xml_diff>
--- a/test/Grades_formatted.xlsx
+++ b/test/Grades_formatted.xlsx
@@ -476,21 +476,21 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Ali</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" t="n">
         <v>88</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" t="n">
         <v>76</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" t="n">
         <v>91</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" t="n">
         <v>85</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -500,21 +500,21 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Sara</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" t="n">
         <v>72</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" t="n">
         <v>85</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" t="n">
         <v>68</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="E3" t="n">
         <v>75</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -524,21 +524,21 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Omar</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" t="n">
         <v>95</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" t="n">
         <v>90</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" t="n">
         <v>74</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" t="n">
         <v>86.3</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -548,21 +548,21 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Lena</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" t="n">
         <v>61</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" t="n">
         <v>55</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" t="n">
         <v>80</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" t="n">
         <v>65.3</v>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -572,21 +572,21 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Jasper</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" t="n">
         <v>78</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" t="n">
         <v>82</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" t="n">
         <v>70</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="E6" t="n">
         <v>76.7</v>
       </c>
       <c r="F6" s="3" t="inlineStr">

</xml_diff>